<commit_message>
Enable admin-style treatment answers from FAQ
- Add 26 FAQ rows from real admin chats (treatment/palliative/rights/pricing/side-effects)
- System prompt: allow general treatment info, forbid individual diagnosis
- Symptom guard: let treatment/price/care questions pass to FAQ
- Groq: max_tokens 512 + trim-to-sentence on length instead of dropping reply

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data ai bot.xlsx
+++ b/data ai bot.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C139"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1642,10 +1642,295 @@
         <v>ขอบคุณที่ติดต่อมานะคะ อยากทราบเพิ่มเติมว่าต้องการข้อมูลด้านใดคะ เช่น อยากตรวจคัดกรอง ต้องการข้อมูลการรักษา หรือมีคนในครอบครัวที่เป็นอยู่คะ</v>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B114" t="str">
+        <v>มะเร็งตับ รักษายังไง มีวิธีไหนบ้าง</v>
+      </c>
+      <c r="C114" t="str">
+        <v>แนวทางการรักษามะเร็งตับขึ้นอยู่กับขนาดก้อน จำนวนก้อน การกระจายของโรค และสภาพการทำงานของตับค่ะ วิธีที่พบบ่อย เช่น การผ่าตัดเอาตับส่วนที่มีก้อนออก, การจี้ทำลายก้อนด้วยความร้อน, การทำ TACE (ปิดท่อน้ำเลี้ยงมะเร็งตับ), ยามุ่งเป้า และยาภูมิคุ้มกันบำบัด คุณหมอจะเป็นผู้ประเมินวิธีที่เหมาะสมกับคนไข้แต่ละท่านค่ะ แนะนำนำผลตรวจเดิมเข้ามาปรึกษาคุณหมอเฉพาะทางนะคะ</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B115" t="str">
+        <v>มะเร็งตับอ่อน รักษาด้วยวิธีใด</v>
+      </c>
+      <c r="C115" t="str">
+        <v>การรักษามะเร็งตับอ่อนขึ้นอยู่กับระยะของโรคและสุขภาพโดยรวมของคนไข้ค่ะ แพทย์อาจใช้หลายวิธีร่วมกัน เช่น การผ่าตัด (มักใช้เมื่อพบระยะแรกและก้อนยังไม่กระจาย), เคมีบำบัด (อาจให้ก่อนผ่าตัดเพื่อลดขนาดก้อน หรือหลังผ่าตัดเพื่อป้องกันเป็นซ้ำ), รังสีรักษา (มักใช้ร่วมกับเคมีบำบัด) และการดูแลแบบประคับประคองเพื่อเพิ่มคุณภาพชีวิต แนะนำนำเอกสารการตรวจวินิจฉัยเดิมมาปรึกษาคุณหมอเพื่อวางแผนร่วมกันค่ะ</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B116" t="str">
+        <v>มะเร็งท่อน้ำดี รักษาได้ไหม ใช้วิธีไหน</v>
+      </c>
+      <c r="C116" t="str">
+        <v>มะเร็งท่อน้ำดีสามารถรักษาได้หลายวิธีค่ะ โดยแพทย์จะพิจารณาจากระยะของโรค ตำแหน่งก้อน การลุกลาม และสภาพร่างกายของคนไข้ แนวทางที่พบบ่อย เช่น การผ่าตัด, เคมีบำบัด, ฉายแสง, การใส่ท่อระบายน้ำดีกรณีมีภาวะอุดตัน และการรักษาแบบมุ่งเป้าหรือภูมิคุ้มกันบำบัดในบางกรณี หากมีผล CT/MRI/ผลชิ้นเนื้อ/ผลเลือด แนะนำนำเข้ามาปรึกษาแพทย์เฉพาะทางเพื่อประเมินแนวทางที่เหมาะสมค่ะ</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B117" t="str">
+        <v>มะเร็งลำไส้ ควรรักษายังไง</v>
+      </c>
+      <c r="C117" t="str">
+        <v>การรักษามะเร็งลำไส้ คุณหมอจะพิจารณาจากระยะของโรค ตำแหน่งก้อน และสุขภาพโดยรวมของคนไข้ค่ะ แนวทางหลักได้แก่ การผ่าตัด (วิธีหลัก โดยเฉพาะระยะเริ่มต้น), เคมีบำบัด (ใช้ร่วมกับผ่าตัดก่อนหรือหลัง), รังสีรักษา (มักใช้กรณีมะเร็งลำไส้ตรง) และยามุ่งเป้าหรือภูมิคุ้มกันบำบัดในกรณีที่โรคกระจาย แนะนำนำผลตรวจเดิมมาปรึกษาคุณหมอเพื่อวางแผนที่เหมาะกับคนไข้ค่ะ</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B118" t="str">
+        <v>มะเร็งโพรงมดลูก รักษายังไง</v>
+      </c>
+      <c r="C118" t="str">
+        <v>แนวทางการรักษามะเร็งโพรงมดลูกขึ้นอยู่กับระยะของโรคและการกระจายตัวค่ะ โดยหลักแพทย์จะใช้ 3 วิธีร่วมกัน ได้แก่ การผ่าตัด (วิธีหลัก มักผ่าตัดมดลูก รังไข่ ท่อนำไข่ และเลาะต่อมน้ำเหลือง หากเป็นระยะเริ่มต้นอาจหายขาดได้), การฉายรังสี (กรณีเสี่ยงกลับมาเป็นซ้ำหรือกระจายรอบมดลูก) และยาเคมีบำบัด/ยามุ่งเป้า (กรณีระยะแพร่กระจาย) คุณหมอจะประเมินให้เหมาะกับคนไข้แต่ละท่านค่ะ</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B119" t="str">
+        <v>มะเร็งต่อมลูกหมาก รักษาได้ไหม</v>
+      </c>
+      <c r="C119" t="str">
+        <v>มะเร็งต่อมลูกหมากปัจจุบันมีแนวทางการรักษาที่ได้ผลดีมาก และมีโอกาสควบคุมโรคได้สูงค่ะ แนวทางมีความยืดหยุ่นขึ้นอยู่กับระยะของโรค ตั้งแต่การทานยา/ฉีดยาฮอร์โมน, การผ่าตัดแผลเล็ก, หรือการฉายแสง คุณหมอจะเลือกวิธีที่ปลอดภัยและเหมาะสมที่สุด แนะนำนำผลตรวจวินิจฉัยและประวัติการรักษาเข้ามาปรึกษาคุณหมอเฉพาะทางเพื่อวางแผนร่วมกันค่ะ</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B120" t="str">
+        <v>มะเร็งปอด ยามุ่งเป้าแบบไหน</v>
+      </c>
+      <c r="C120" t="str">
+        <v>การจะใช้ยามุ่งเป้าในมะเร็งปอดได้ ผู้ป่วยต้องผ่านการตรวจยีนกลายพันธุ์ (Biomarker Testing) จากชิ้นเนื้อหรือผลเลือดก่อนค่ะ หากพบการกลายพันธุ์ที่ตรงกับยา จึงจะสามารถใช้ยามุ่งเป้าตัวนั้นได้ แนะนำนำผลตรวจเข้ามาปรึกษาคุณหมอเฉพาะทางเพื่อประเมินค่ะ</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="str">
+        <v>แนวทางการรักษา</v>
+      </c>
+      <c r="B121" t="str">
+        <v>มะเร็งเต้านมระยะ 4 ลามไปกระดูก/ตับ/ต่อมน้ำเหลือง รักษาได้ไหม</v>
+      </c>
+      <c r="C121" t="str">
+        <v>ยังรักษาได้ค่ะ กรณีมะเร็งเต้านมระยะที่ 4 ที่มีการกระจาย เป้าหมายการรักษามักเป็นการควบคุมโรค ชะลอการลุกลาม ลดอาการ และให้คนไข้มีคุณภาพชีวิตที่ดี ปัจจุบันมีทั้งยาเคมีบำบัด ยามุ่งเป้า และยาฮอร์โมน ซึ่งช่วยควบคุมโรคได้อย่างมีประสิทธิภาพ แนะนำนำประวัติการรักษาเดิมเข้ามาปรึกษาคุณหมอเพื่อวางแผนที่เหมาะกับคนไข้ค่ะ</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="str">
+        <v>ประคับประคอง</v>
+      </c>
+      <c r="B122" t="str">
+        <v>การรักษาแบบประคับประคองคือจุดสิ้นสุดของการรักษาแล้วหรือ</v>
+      </c>
+      <c r="C122" t="str">
+        <v>การรักษาแบบประคับประคองไม่ได้หมายความว่าเป็นจุดสิ้นสุดของการรักษานะคะ แต่เป็นการดูแลเพื่อควบคุมอาการ ลดความเจ็บปวด และช่วยให้ผู้ป่วยมีคุณภาพชีวิตที่ดีที่สุด ในบางกรณีแพทย์อาจพิจารณาร่วมกับการรักษาอื่นตามความเหมาะสมของผู้ป่วยแต่ละรายค่ะ</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="str">
+        <v>ประคับประคอง</v>
+      </c>
+      <c r="B123" t="str">
+        <v>ผู้ป่วยระยะสุดท้าย/ประคับประคอง อยากปรึกษาการดูแล</v>
+      </c>
+      <c r="C123" t="str">
+        <v>ขอส่งกำลังใจให้คนไข้และครอบครัวนะคะ แม้จะอยู่ในช่วงประคับประคอง ทางการแพทย์ยังมีวิธีช่วยควบคุมอาการและดูแลให้คนไข้ทรมานน้อยลง มีคุณภาพชีวิตที่ดีขึ้นได้ค่ะ ศูนย์ชีวารักษ์มีแนวทางดูแลแบบประคับประคอง หากสนใจสามารถนำประวัติการรักษาของคนไข้เข้ามาปรึกษาคุณหมอเพื่อเป็นทางเลือกในการดูแลได้ค่ะ เจ้าหน้าที่ทำนัดให้ได้เลยนะคะ</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="str">
+        <v>ประคับประคอง</v>
+      </c>
+      <c r="B124" t="str">
+        <v>ยาภูมิคุ้มกันบำบัดช่วยได้ไหมในผู้ป่วยระยะท้าย</v>
+      </c>
+      <c r="C124" t="str">
+        <v>การประเมินแนวทางการรักษาคุณหมอจะเป็นผู้ประเมินให้ค่ะ เสมือนการออกแบบการรักษาให้เหมาะกับสภาพร่างกายและรอยโรคของผู้ป่วยแต่ละท่านโดยเฉพาะ ข้อมูลส่วนบุคคลและประวัติการรักษาจึงจำเป็นอย่างยิ่ง แนะนำนำเอกสารหรือประวัติการรักษาเข้าพบแพทย์ผู้เชี่ยวชาญเพื่อร่วมปรึกษาและวางแผนแนวทางที่มีประสิทธิภาพสูงสุดร่วมกันค่ะ</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="str">
+        <v>สิทธิ์การรักษา</v>
+      </c>
+      <c r="B125" t="str">
+        <v>ใช้สิทธิ์บัตรทอง 30 บาท ประกันสังคม ข้าราชการ ได้ไหม</v>
+      </c>
+      <c r="C125" t="str">
+        <v>ขอเรียนชี้แจงนะคะ ขณะนี้ศูนย์มะเร็งชีวารักษ์ให้บริการสำหรับการชำระเงินสด หรือประกันชีวิต/ประกันสุขภาพที่ครอบคลุมค่ารักษาเท่านั้นค่ะ ส่วนสิทธิ์ภาครัฐ (บัตรทอง/ประกันสังคม/ข้าราชการ) ศูนย์ยังไม่ได้เข้าร่วมระบบเบิกจ่าย จึงยังไม่สามารถใช้สิทธิ์ดังกล่าวได้ในตอนนี้นะคะ</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="str">
+        <v>สิทธิ์การรักษา</v>
+      </c>
+      <c r="B126" t="str">
+        <v>เบิกกรมบัญชีกลางได้ไหม เป็นข้าราชการ</v>
+      </c>
+      <c r="C126" t="str">
+        <v>กรณีเข้ารับการรักษาโรคทั่วไปแบบผู้ป่วยนอก (OPD) หรือผู้ป่วยใน (IPD) ที่โรงพยาบาลเอกชนโดยไม่มีข้อบ่งชี้ฉุกเฉิน จะเบิกคืนจากกรมบัญชีกลางไม่ได้ค่ะ ต้องชำระเองหรือใช้ประกันสุขภาพส่วนบุคคลแทน และที่ศูนย์ชีวารักษ์ยังไม่รองรับสิทธิ์ข้าราชการนะคะ รองรับเฉพาะเงินสดและประกันชีวิต/ประกันสุขภาพค่ะ</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="str">
+        <v>สิทธิ์การรักษา</v>
+      </c>
+      <c r="B127" t="str">
+        <v>ใช้สิทธิ์ประกันกลุ่มแบบ IPD ได้ไหม คุณหมอให้แอดมิทได้ไหม</v>
+      </c>
+      <c r="C127" t="str">
+        <v>การพิจารณาให้แอดมิทนอนโรงพยาบาล (IPD) ขึ้นอยู่กับดุลยพินิจของคุณหมอเจ้าของไข้ โดยประเมินจากความจำเป็นทางการแพทย์เป็นหลักค่ะ เช่น สูตรยาที่ต้องหยดนานหลายชั่วโมง หรือต้องมอนิเตอร์อาการข้างเคียงใกล้ชิด หรือสภาพร่างกายคนไข้มีความเสี่ยงหากกลับบ้านทันที คุณหมอจะออกใบรับรองและบันทึกประวัติให้ตรงตามความเป็นจริงของโรค เพื่อให้สอดคล้องกับเกณฑ์การเคลมของบริษัทประกันค่ะ</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="str">
+        <v>ค่าใช้จ่าย</v>
+      </c>
+      <c r="B128" t="str">
+        <v>ค่ารักษามะเร็งแพงไหม ประมาณเท่าไร</v>
+      </c>
+      <c r="C128" t="str">
+        <v>ค่ารักษามะเร็งขึ้นอยู่กับหลายปัจจัยค่ะ เช่น ชนิดของมะเร็ง ระยะโรค และแนวทางการรักษาที่คุณหมอเลือก หากมีผลตรวจหรือเอกสารเดิม แนะนำนำมาด้วยนะคะ จะช่วยให้คุณหมอวางแผนรักษาและทางพยาบาลประเมินค่าใช้จ่ายเบื้องต้นให้ได้ค่ะ สะดวกให้ชื่อและเบอร์ติดต่อกลับเพื่อทำนัดพบคุณหมอไหมคะ</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="str">
+        <v>ค่าใช้จ่าย</v>
+      </c>
+      <c r="B129" t="str">
+        <v>ค่าปรึกษาพบแพทย์ครั้งแรกเท่าไร</v>
+      </c>
+      <c r="C129" t="str">
+        <v>ค่าใช้จ่ายในการเข้าพบและปรึกษาคุณหมอเฉพาะทางครั้งแรกเริ่มต้นประมาณ 2,000 บาทค่ะ แนะนำนำผลตรวจวินิจฉัยและประวัติการรักษาเดิมมาด้วย เพื่อให้คุณหมอวางแผนแนวทางการรักษาได้แม่นยำค่ะ</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="str">
+        <v>ค่าใช้จ่าย</v>
+      </c>
+      <c r="B130" t="str">
+        <v>ค่าตรวจคัดกรองมะเร็งเต้านมราคาเท่าไร</v>
+      </c>
+      <c r="C130" t="str">
+        <v>แพ็กเกจตรวจ Mammogram แบบ 3 มิติ (3D) แถมฟรี Ultrasound เต้านม ราคา 3,500 บาทค่ะ คุ้มค่ามาก เพราะ Mammogram 3 มิติเห็นรายละเอียดรอยโรคเล็ก ๆ ได้ชัดกว่าปกติ และมี Ultrasound เต้านมควบคู่ไปด้วยค่ะ</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="str">
+        <v>การตรวจคัดกรอง</v>
+      </c>
+      <c r="B131" t="str">
+        <v>ตรวจแมมโมแกรม 3D เจ็บไหม</v>
+      </c>
+      <c r="C131" t="str">
+        <v>จะรู้สึกตึงและเจ็บหน่วง ๆ ปานกลาง แต่เจ็บแค่ไม่กี่วินาทีต่อท่าค่ะ เพราะเจ้าหน้าที่ต้องใช้แผ่นกดเนื้อเต้านมให้แผ่ออกเพื่อให้เห็นรอยโรคชัด ระบบ 3D จะถ่ายหลายมุม (Tomosynthesis) เห็นเนื้อนมเป็นชั้น ๆ และมักกดสั้นลงนุ่มนวลกว่าระบบเก่า แต่ละท่ากดประมาณ 5-10 วินาที ถ่ายทั้งหมดประมาณ 4 ท่า ซ้าย-ขวา ส่วน Ultrasound เต้านมจะทาเจลแล้วใช้หัวตรวจเลื่อนบนผิว ไม่เจ็บค่ะ</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="str">
+        <v>การตรวจคัดกรอง</v>
+      </c>
+      <c r="B132" t="str">
+        <v>ตรวจเลือดเช็คมะเร็งได้ไหม ค่าใช้จ่ายเท่าไร</v>
+      </c>
+      <c r="C132" t="str">
+        <v>ตรวจเลือดเช็คความเสี่ยงมะเร็ง (สารบ่งชี้มะเร็ง) ทำได้ค่ะ แต่ขอแนะนำเบื้องต้นว่าการตรวจเลือดจะดูแนวโน้มความเสี่ยงเท่านั้น ค่าเลือดสูงไม่ได้แปลว่าเป็นมะเร็งเสมอไป เพราะภาวะอักเสบหรือพฤติกรรมบางอย่างก็ทำให้ค่าขยับได้ เพื่อความแม่นยำแนะนำตรวจเลือดควบคู่การตรวจเฉพาะทางตามช่วงอายุ เช่น อัลตราซาวด์ช่องท้อง หรือคัดกรองมะเร็งปากมดลูก/เต้านม หากมีความกังวลด้านใด แนะนำเข้ามาเช็คสุขภาพแต่เนิ่น ๆ ตรวจเร็วเจอไว รักษาได้ค่ะ</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="str">
+        <v>ผลข้างเคียง</v>
+      </c>
+      <c r="B133" t="str">
+        <v>คีโมมีผลข้างเคียงไหม</v>
+      </c>
+      <c r="C133" t="str">
+        <v>ยาเคมีบำบัดออกฤทธิ์กับเซลล์ที่เจริญเติบโตเร็วทั้งเซลล์ปกติและเซลล์มะเร็งค่ะ จึงส่งผลข้างเคียงต่อเซลล์ปกติที่โตเร็ว เช่น เซลล์เม็ดเลือด ผิวหนัง รูขุมขน และเยื่อบุทางเดินอาหาร ผลข้างเคียงที่พบบ่อย เช่น อ่อนเพลีย เหนื่อยล้า คลื่นไส้ อาเจียน เบื่ออาหาร ผมร่วง ทั้งนี้อาการและความรุนแรงแตกต่างกันในแต่ละคนค่ะ</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="str">
+        <v>ผลข้างเคียง</v>
+      </c>
+      <c r="B134" t="str">
+        <v>มือเท้าชาหลังทำคีโม ทำยังไงดี</v>
+      </c>
+      <c r="C134" t="str">
+        <v>อาการชาปลายมือปลายเท้าหลังรับคีโมเป็นผลข้างเคียงที่พบได้บ่อยค่ะ เกิดจากตัวยาส่งผลต่อเส้นประสาทส่วนปลายชั่วคราว ส่วนใหญ่จะค่อย ๆ ดีขึ้นหลังสิ้นสุดการรักษา วิธีดูแลตัวเองเบื้องต้น เช่น ระวังของมีคมและความร้อน (เช็คอุณหภูมิน้ำก่อนใช้), สวมรองเท้านุ่มกระชับตลอดเวลาแม้อยู่บ้าน, นวดมือเท้าเบา ๆ หรือแช่น้ำอุ่น (เลี่ยงน้ำร้อนจัด), และขยับนิ้วมือนิ้วเท้าหรือออกกำลังกายเบา ๆ บ่อย ๆ ค่ะ</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="str">
+        <v>ผลข้างเคียง</v>
+      </c>
+      <c r="B135" t="str">
+        <v>กินวิตามิน/อาหารเสริมระหว่างทำคีโมได้ไหม</v>
+      </c>
+      <c r="C135" t="str">
+        <v>แนะนำให้เซฟรูปหรือถือกระปุกวิตามินตัวจริงไปให้คุณหมอเจ้าของไข้ดูในวันนัดรับยาครั้งต่อไปนะคะ เพราะคุณหมอจะเช็คสูตรยาคีโมที่ได้รับปัจจุบันควบคู่กับส่วนประกอบของวิตามินได้อย่างแม่นยำและปลอดภัยที่สุด ควรแจ้งแพทย์ทุกครั้งหากทานวิตามิน อาหารเสริม หรือสมุนไพรเพิ่ม เพราะบางชนิดอาจส่งผลต่อการรักษาค่ะ</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="str">
+        <v>การเตรียมตัว</v>
+      </c>
+      <c r="B136" t="str">
+        <v>ต้องเตรียมตัวยังไงก่อนทำคีโม</v>
+      </c>
+      <c r="C136" t="str">
+        <v>ก่อนเข้ารับการรักษาแนะนำเตรียมตัวเบื้องต้นดังนี้ค่ะ พักผ่อนให้เพียงพอและทานอาหารอ่อนย่อยง่าย, เตรียมประวัติการรักษา ยาประจำตัว หรือผลตรวจเดิม (ถ้ามี), แจ้งโรคประจำตัวและประวัติแพ้ยาแก่แพทย์ทุกครั้ง, หากมีประกันสุขภาพ/ประกันชีวิตนำเอกสารมาให้เจ้าหน้าที่ตรวจสอบสิทธิ์ได้ และกรณีมีการตรวจพิเศษบางชนิดอาจต้องงดน้ำงดอาหาร เจ้าหน้าที่จะแจ้งล่วงหน้าค่ะ</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="str">
+        <v>การดูแลหลังผ่าตัด</v>
+      </c>
+      <c r="B137" t="str">
+        <v>หลังผ่าตัดลำไส้ใหญ่ นานไหมกว่าจะออกกำลังกายได้</v>
+      </c>
+      <c r="C137" t="str">
+        <v>ระยะเวลาเริ่มออกกำลังกายหลังผ่าตัดลำไส้ใหญ่แตกต่างกันตามชนิดการผ่าตัดและการฟื้นตัวของแต่ละท่านค่ะ ช่วงแรกแนะนำเริ่มจากเดินเบา ๆ เพื่อกระตุ้นการไหลเวียนเลือดและช่วยฟื้นตัว ส่วนการออกกำลังที่ใช้แรงมาก ยกของหนัก หรือเกร็งหน้าท้อง มักแนะนำให้รอประมาณ 4-8 สัปดาห์ หรือจนกว่าจะได้รับคำแนะนำจากแพทย์ผู้รักษาค่ะ</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="str">
+        <v>ทั่วไป</v>
+      </c>
+      <c r="B138" t="str">
+        <v>มะเร็งรักษาหายไหม มีคนหายไหม</v>
+      </c>
+      <c r="C138" t="str">
+        <v>โอกาสรักษาหายขึ้นอยู่กับหลายปัจจัยร่วมกันค่ะ เช่น ชนิดของมะเร็ง ระยะของโรคเมื่อตรวจพบ และสภาพร่างกายโดยรวมของผู้ป่วย ปัจจุบันเทคโนโลยีการรักษามะเร็งก้าวหน้าไปมาก ทั้งการผ่าตัดส่องกล้อง เคมีบำบัดสูตรใหม่ รังสีรักษาที่แม่นยำ ยามุ่งเป้า และภูมิคุ้มกันบำบัด หากตรวจพบระยะเริ่มต้นและรักษาต่อเนื่องตามแผนของแพทย์ ก็มีโอกาสสูงที่จะควบคุมโรคได้สำเร็จหรือเข้าสู่ภาวะสงบของโรค จนกลับมาใช้ชีวิตปกติได้ค่ะ</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="str">
+        <v>การนัดหมาย</v>
+      </c>
+      <c r="B139" t="str">
+        <v>อยากปรึกษาหมอ/ขอความเห็นที่สอง (Second Opinion) ต้องเตรียมอะไร</v>
+      </c>
+      <c r="C139" t="str">
+        <v>เพื่อให้คุณหมอประเมินแนวทางและค่าใช้จ่ายได้แม่นยำที่สุด แนะนำเตรียมเอกสารประวัติการรักษาเดิมมาในวันนัดดังนี้ค่ะ ผลตรวจชิ้นเนื้อ (Pathology Report), ใบสรุปการรักษาหรือประวัติการให้ยา/ผ่าตัด/ฉายแสงเดิม, ผลตรวจเลือดล่าสุด, แผ่น CD หรือ Flash Drive ผลตรวจทางรังสี (CT Scan/MRI/PET Scan) พร้อมใบรายงานผล, ยาประจำตัวที่ทานอยู่ และบัตรประชาชนตัวจริง สามารถถ่ายรูปเอกสารส่งเข้ามาในแชท และให้ชื่อ-เบอร์ติดต่อ เจ้าหน้าที่จะประสานนัดคิวพบคุณหมอเฉพาะทางให้ค่ะ</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C113"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C139"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Consolidate breast screening price into one consistent 3-tier answer
</commit_message>
<xml_diff>
--- a/data ai bot.xlsx
+++ b/data ai bot.xlsx
@@ -872,15 +872,19 @@
         <v>แมมโมแกรมคือการเอกซเรย์เต้านมด้วยรังสีขนาดต่ำ เหมาะตรวจก้อนที่มองไม่เห็นจากภายนอก ส่วนอัลตร้าซาวด์ใช้คลื่นเสียงแยกแยะก้อนน้ำและก้อนเนื้อ แนะนำทำคู่กันเพื่อความแม่นยำสูงสุด</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" xml:space="preserve">
       <c r="A44" t="str">
         <v>มะเร็งเต้านม</v>
       </c>
       <c r="B44" t="str">
         <v>ราคาตรวจแมมโมแกรมเท่าไร</v>
       </c>
-      <c r="C44" t="str">
-        <v>ตรวจด้วยอัลตร้าซาวด์ ราคา 1,700 บาท / แมมโมแกรมดิจิตอล + อัลตร้าซาวด์ ราคา 2,500 บาท</v>
+      <c r="C44" t="str" xml:space="preserve">
+        <v xml:space="preserve">ราคาตรวจคัดกรองมะเร็งเต้านม มีให้เลือกดังนี้ค่ะ
+• อัลตร้าซาวด์เต้านม 1,700 บาท
+• ดิจิตอลแมมโมแกรม + อัลตร้าซาวด์ 2,500 บาท
+• แมมโมแกรม 3 มิติ (3D) + อัลตร้าซาวด์ 3,500 บาท
+ราคาอาจเปลี่ยนแปลงตามโปรโมชั่น สอบถามราคาล่าสุดโทร 063-816-6058 ค่ะ</v>
       </c>
     </row>
     <row r="45">
@@ -1180,15 +1184,19 @@
         <v>Thin Prep: 1,650 บาท / Thin Prep + HPV DNA: 2,900 บาท</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" xml:space="preserve">
       <c r="A72" t="str">
         <v>แพ็กเกจ/ราคา</v>
       </c>
       <c r="B72" t="str">
         <v>ตรวจคัดกรองมะเร็งเต้านมราคาเท่าไร</v>
       </c>
-      <c r="C72" t="str">
-        <v>อัลตร้าซาวด์: 1,700 บาท / ดิจิตอลแมมโมแกรม + อัลตร้าซาวด์: 2,500 บาท</v>
+      <c r="C72" t="str" xml:space="preserve">
+        <v xml:space="preserve">ราคาตรวจคัดกรองมะเร็งเต้านม มีให้เลือกดังนี้ค่ะ
+• อัลตร้าซาวด์เต้านม 1,700 บาท
+• ดิจิตอลแมมโมแกรม + อัลตร้าซาวด์ 2,500 บาท
+• แมมโมแกรม 3 มิติ (3D) + อัลตร้าซาวด์ 3,500 บาท
+ราคาอาจเปลี่ยนแปลงตามโปรโมชั่น สอบถามราคาล่าสุดโทร 063-816-6058 ค่ะ</v>
       </c>
     </row>
     <row r="73">
@@ -1818,15 +1826,19 @@
         <v>ค่าใช้จ่ายในการเข้าพบและปรึกษาคุณหมอเฉพาะทางครั้งแรกเริ่มต้นประมาณ 2,000 บาทค่ะ แนะนำนำผลตรวจวินิจฉัยและประวัติการรักษาเดิมมาด้วย เพื่อให้คุณหมอวางแผนแนวทางการรักษาได้แม่นยำค่ะ</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" xml:space="preserve">
       <c r="A130" t="str">
         <v>ค่าใช้จ่าย</v>
       </c>
       <c r="B130" t="str">
         <v>ค่าตรวจคัดกรองมะเร็งเต้านมราคาเท่าไร</v>
       </c>
-      <c r="C130" t="str">
-        <v>แพ็กเกจตรวจ Mammogram แบบ 3 มิติ (3D) แถมฟรี Ultrasound เต้านม ราคา 3,500 บาทค่ะ คุ้มค่ามาก เพราะ Mammogram 3 มิติเห็นรายละเอียดรอยโรคเล็ก ๆ ได้ชัดกว่าปกติ และมี Ultrasound เต้านมควบคู่ไปด้วยค่ะ</v>
+      <c r="C130" t="str" xml:space="preserve">
+        <v xml:space="preserve">ราคาตรวจคัดกรองมะเร็งเต้านม มีให้เลือกดังนี้ค่ะ
+• อัลตร้าซาวด์เต้านม 1,700 บาท
+• ดิจิตอลแมมโมแกรม + อัลตร้าซาวด์ 2,500 บาท
+• แมมโมแกรม 3 มิติ (3D) + อัลตร้าซาวด์ 3,500 บาท
+ราคาอาจเปลี่ยนแปลงตามโปรโมชั่น สอบถามราคาล่าสุดโทร 063-816-6058 ค่ะ</v>
       </c>
     </row>
     <row r="131">

</xml_diff>

<commit_message>
Add FAQ: explain 3 breast screening options
</commit_message>
<xml_diff>
--- a/data ai bot.xlsx
+++ b/data ai bot.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C139"/>
+  <dimension ref="A1:C140"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1940,9 +1940,24 @@
         <v>เพื่อให้คุณหมอประเมินแนวทางและค่าใช้จ่ายได้แม่นยำที่สุด แนะนำเตรียมเอกสารประวัติการรักษาเดิมมาในวันนัดดังนี้ค่ะ ผลตรวจชิ้นเนื้อ (Pathology Report), ใบสรุปการรักษาหรือประวัติการให้ยา/ผ่าตัด/ฉายแสงเดิม, ผลตรวจเลือดล่าสุด, แผ่น CD หรือ Flash Drive ผลตรวจทางรังสี (CT Scan/MRI/PET Scan) พร้อมใบรายงานผล, ยาประจำตัวที่ทานอยู่ และบัตรประชาชนตัวจริง สามารถถ่ายรูปเอกสารส่งเข้ามาในแชท และให้ชื่อ-เบอร์ติดต่อ เจ้าหน้าที่จะประสานนัดคิวพบคุณหมอเฉพาะทางให้ค่ะ</v>
       </c>
     </row>
+    <row r="140" xml:space="preserve">
+      <c r="A140" t="str">
+        <v>มะเร็งเต้านม</v>
+      </c>
+      <c r="B140" t="str">
+        <v>3 แบบตรวจเต้านม ต่างกันยังไง อัลตร้าซาวด์ ดิจิตอลแมมโมแกรม 3D</v>
+      </c>
+      <c r="C140" t="str" xml:space="preserve">
+        <v xml:space="preserve">แต่ละแบบต่างกันดังนี้ค่ะ
+• อัลตร้าซาวด์เต้านม ใช้คลื่นเสียง ไม่เจ็บ ไม่มีรังสี เหมาะแยกก้อนน้ำกับก้อนเนื้อ และเหมาะกับผู้หญิงอายุน้อยที่เนื้อนมแน่น
+• ดิจิตอลแมมโมแกรม (2 มิติ) เอกซเรย์เต้านมด้วยรังสีขนาดต่ำ เห็นก้อนและจุดหินปูนเล็ก ๆ ที่คลำไม่เจอ ภาพเป็นภาพแบน 2 มิติ
+• แมมโมแกรม 3 มิติ (3D/Tomosynthesis) ถ่ายหลายมุมแล้วประกอบเป็นภาพเนื้อนมเป็นชั้น ๆ เห็นรอยโรคชัดกว่า 2 มิติ ลดโอกาสเนื้อนมหนาบังก้อน แม่นยำกว่า
+โดยทั่วไปแนะนำตรวจแมมโมแกรมคู่กับอัลตร้าซาวด์เพื่อความแม่นยำสูงสุดค่ะ คุณหมอจะแนะนำแบบที่เหมาะกับคุณให้ สอบถามเพิ่มเติมโทร 063-816-6058 ค่ะ</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C139"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C140"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>